<commit_message>
feat: implement notas_custom mode for drawing note tables manually
</commit_message>
<xml_diff>
--- a/backend/templates/CAF - BRIGHTEC - 2026.02 - plantilla-balance (1).xlsx
+++ b/backend/templates/CAF - BRIGHTEC - 2026.02 - plantilla-balance (1).xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bryal\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bryal\OneDrive\Escritorio\AutoTeaser\AUTOTEASER\backend\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7754BD21-D104-4628-86C9-0406C6992820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7D41A13-59DF-472C-B1A9-372F19D47CEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3855" yWindow="4185" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Balance" sheetId="1" r:id="rId1"/>
@@ -2467,16 +2467,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="168" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2519,23 +2509,33 @@
     <xf numFmtId="0" fontId="22" fillId="5" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="26" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="43" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="13" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -2879,39 +2879,41 @@
       <c r="A3" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="B3" s="324"/>
-      <c r="C3" s="325"/>
-      <c r="D3" s="326">
+      <c r="B3" s="320">
+        <v>2023</v>
+      </c>
+      <c r="C3" s="321"/>
+      <c r="D3" s="322">
         <f>B3+1</f>
-        <v>1</v>
-      </c>
-      <c r="E3" s="325"/>
-      <c r="F3" s="317">
+        <v>2024</v>
+      </c>
+      <c r="E3" s="321"/>
+      <c r="F3" s="313">
         <f>D3+1</f>
-        <v>2</v>
-      </c>
-      <c r="G3" s="318"/>
-      <c r="H3" s="327" t="str">
+        <v>2025</v>
+      </c>
+      <c r="G3" s="314"/>
+      <c r="H3" s="323" t="str">
         <f>F3+1&amp;" "&amp;"("&amp;IF('Edo de resultados'!K2=1,"Enero",IF('Edo de resultados'!K2=2,"Febrero",IF('Edo de resultados'!K2=3,"Marzo",IF('Edo de resultados'!K2=4,"Abril",IF('Edo de resultados'!K2=5,"Mayo",IF('Edo de resultados'!K2=6,"Junio",IF('Edo de resultados'!K2=7,"Julio",IF('Edo de resultados'!K2=8,"Agosto",IF('Edo de resultados'!K2=9,"Septiembre",IF('Edo de resultados'!K2=10,"Octubre",IF('Edo de resultados'!K2=11,"Noviembre",IF('Edo de resultados'!K2=12,"Diciembre","INCORRECTO"))))))))))))&amp;")"</f>
-        <v>3 (INCORRECTO)</v>
-      </c>
-      <c r="I3" s="325"/>
+        <v>2026 (INCORRECTO)</v>
+      </c>
+      <c r="I3" s="321"/>
       <c r="J3" s="4"/>
       <c r="K3" s="5" t="str">
         <f>"Razones"&amp;" "&amp;B3</f>
-        <v xml:space="preserve">Razones </v>
+        <v>Razones 2023</v>
       </c>
       <c r="L3" s="6" t="str">
         <f>"Razones"&amp;" "&amp;B3+1</f>
-        <v>Razones 1</v>
+        <v>Razones 2024</v>
       </c>
       <c r="M3" s="7" t="str">
         <f>"Razones"&amp;" "&amp;B3+2</f>
-        <v>Razones 2</v>
+        <v>Razones 2025</v>
       </c>
       <c r="N3" s="8" t="str">
         <f>"Razones"&amp;" "&amp;B3+3</f>
-        <v>Razones 3</v>
+        <v>Razones 2026</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4445,17 +4447,17 @@
       </c>
     </row>
     <row r="47" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="321" t="s">
+      <c r="A47" s="317" t="s">
         <v>119</v>
       </c>
-      <c r="B47" s="320"/>
-      <c r="C47" s="320"/>
-      <c r="D47" s="320"/>
-      <c r="E47" s="322"/>
-      <c r="F47" s="319"/>
-      <c r="G47" s="320"/>
-      <c r="H47" s="323"/>
-      <c r="I47" s="322"/>
+      <c r="B47" s="316"/>
+      <c r="C47" s="316"/>
+      <c r="D47" s="316"/>
+      <c r="E47" s="318"/>
+      <c r="F47" s="315"/>
+      <c r="G47" s="316"/>
+      <c r="H47" s="319"/>
+      <c r="I47" s="318"/>
       <c r="J47" s="21"/>
       <c r="K47" s="40" t="e">
         <f>B70/B82</f>
@@ -5270,17 +5272,17 @@
       <c r="J72" s="13"/>
     </row>
     <row r="73" spans="1:15" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="321" t="s">
+      <c r="A73" s="317" t="s">
         <v>154</v>
       </c>
-      <c r="B73" s="320"/>
-      <c r="C73" s="320"/>
-      <c r="D73" s="320"/>
-      <c r="E73" s="322"/>
-      <c r="F73" s="319"/>
-      <c r="G73" s="320"/>
-      <c r="H73" s="323"/>
-      <c r="I73" s="322"/>
+      <c r="B73" s="316"/>
+      <c r="C73" s="316"/>
+      <c r="D73" s="316"/>
+      <c r="E73" s="318"/>
+      <c r="F73" s="315"/>
+      <c r="G73" s="316"/>
+      <c r="H73" s="319"/>
+      <c r="I73" s="318"/>
       <c r="J73" s="13"/>
       <c r="K73" s="125" t="s">
         <v>155</v>
@@ -13552,31 +13554,31 @@
       <c r="A3" s="176" t="s">
         <v>189</v>
       </c>
-      <c r="B3" s="332">
+      <c r="B3" s="328">
         <f>Balance!B3</f>
-        <v>0</v>
-      </c>
-      <c r="C3" s="329"/>
-      <c r="D3" s="333">
+        <v>2023</v>
+      </c>
+      <c r="C3" s="325"/>
+      <c r="D3" s="329">
         <f>B3+1</f>
-        <v>1</v>
-      </c>
-      <c r="E3" s="329"/>
-      <c r="F3" s="328">
+        <v>2024</v>
+      </c>
+      <c r="E3" s="325"/>
+      <c r="F3" s="324">
         <f>D3+1</f>
-        <v>2</v>
-      </c>
-      <c r="G3" s="329"/>
-      <c r="H3" s="334" t="str">
+        <v>2025</v>
+      </c>
+      <c r="G3" s="325"/>
+      <c r="H3" s="330" t="str">
         <f>F3+1&amp;" "&amp;"("&amp;IF(K2=1,"enero",IF(K2=2,"febrero",IF(K2=3,"marzo",IF(K2=4,"abril",IF(K2=5,"mayo",IF(K2=6,"junio",IF(K2=7,"julio",IF(K2=8,"agosto",IF(K2=9,"septiembre",IF(K2=10,"octubre",IF(K2=11,"noviembre",IF(K2=12,"diciembre","INCORRECTO"))))))))))))&amp;")"</f>
-        <v>3 (INCORRECTO)</v>
-      </c>
-      <c r="I3" s="331"/>
-      <c r="J3" s="330" t="str">
+        <v>2026 (INCORRECTO)</v>
+      </c>
+      <c r="I3" s="327"/>
+      <c r="J3" s="326" t="str">
         <f>F3+1&amp;" "&amp;"anualizado"</f>
-        <v>3 anualizado</v>
-      </c>
-      <c r="K3" s="331"/>
+        <v>2026 anualizado</v>
+      </c>
+      <c r="K3" s="327"/>
       <c r="L3" s="151"/>
       <c r="M3" s="151"/>
       <c r="N3" s="151"/>
@@ -42037,21 +42039,21 @@
       <c r="B1" s="240" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="313">
+      <c r="C1" s="331">
         <f>Balance!B3</f>
-        <v>0</v>
-      </c>
-      <c r="D1" s="314"/>
-      <c r="E1" s="316">
+        <v>2023</v>
+      </c>
+      <c r="D1" s="332"/>
+      <c r="E1" s="334">
         <f>C1+1</f>
-        <v>1</v>
-      </c>
-      <c r="F1" s="314"/>
-      <c r="G1" s="315">
+        <v>2024</v>
+      </c>
+      <c r="F1" s="332"/>
+      <c r="G1" s="333">
         <f>E1+1</f>
-        <v>2</v>
-      </c>
-      <c r="H1" s="314"/>
+        <v>2025</v>
+      </c>
+      <c r="H1" s="332"/>
       <c r="J1" s="241" t="s">
         <v>1</v>
       </c>
@@ -42083,19 +42085,19 @@
       </c>
       <c r="J2" s="244">
         <f>K2-1</f>
-        <v>0</v>
+        <v>2023</v>
       </c>
       <c r="K2" s="244">
         <f>E1</f>
-        <v>1</v>
+        <v>2024</v>
       </c>
       <c r="L2" s="244">
         <f>K2+1</f>
-        <v>2</v>
+        <v>2025</v>
       </c>
       <c r="M2" s="244">
         <f>L2+1</f>
-        <v>3</v>
+        <v>2026</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.25">
@@ -44533,17 +44535,17 @@
         <f>Balance!D1</f>
         <v>BRIGHTEC ENERGY DYNAMICS S DE RL DE CV</v>
       </c>
-      <c r="M1" s="337" t="s">
+      <c r="M1" s="335" t="s">
         <v>215</v>
       </c>
       <c r="N1" s="336"/>
       <c r="O1" s="336"/>
-      <c r="Q1" s="337" t="s">
+      <c r="Q1" s="335" t="s">
         <v>216</v>
       </c>
       <c r="R1" s="336"/>
       <c r="S1" s="336"/>
-      <c r="U1" s="337" t="s">
+      <c r="U1" s="335" t="s">
         <v>217</v>
       </c>
       <c r="V1" s="336"/>
@@ -44555,17 +44557,17 @@
         <f>'Edo de resultados'!K2</f>
         <v>0</v>
       </c>
-      <c r="M2" s="335" t="s">
+      <c r="M2" s="339" t="s">
         <v>218</v>
       </c>
       <c r="N2" s="336"/>
       <c r="O2" s="336"/>
-      <c r="Q2" s="335" t="s">
+      <c r="Q2" s="339" t="s">
         <v>218</v>
       </c>
       <c r="R2" s="336"/>
       <c r="S2" s="336"/>
-      <c r="U2" s="335" t="s">
+      <c r="U2" s="339" t="s">
         <v>218</v>
       </c>
       <c r="V2" s="336"/>
@@ -44575,29 +44577,29 @@
       <c r="A3" s="262" t="s">
         <v>189</v>
       </c>
-      <c r="B3" s="338">
+      <c r="B3" s="341">
         <f>'Edo de resultados'!B3:C3</f>
-        <v>0</v>
-      </c>
-      <c r="C3" s="314"/>
-      <c r="D3" s="340">
+        <v>2023</v>
+      </c>
+      <c r="C3" s="332"/>
+      <c r="D3" s="337">
         <f>'Edo de resultados'!D3:E3</f>
-        <v>1</v>
-      </c>
-      <c r="E3" s="314"/>
-      <c r="F3" s="339">
+        <v>2024</v>
+      </c>
+      <c r="E3" s="332"/>
+      <c r="F3" s="340">
         <f>'Edo de resultados'!F3:G3</f>
-        <v>2</v>
-      </c>
-      <c r="G3" s="314"/>
-      <c r="H3" s="341" t="str">
+        <v>2025</v>
+      </c>
+      <c r="G3" s="332"/>
+      <c r="H3" s="338" t="str">
         <f>'Edo de resultados'!H3:I3</f>
-        <v>3 (INCORRECTO)</v>
-      </c>
-      <c r="I3" s="314"/>
+        <v>2026 (INCORRECTO)</v>
+      </c>
+      <c r="I3" s="332"/>
       <c r="J3" s="263" t="str">
         <f>'Edo de resultados'!J3:K3</f>
-        <v>3 anualizado</v>
+        <v>2026 anualizado</v>
       </c>
       <c r="K3" s="264"/>
       <c r="M3" s="265" t="s">
@@ -45416,12 +45418,12 @@
       <c r="I19" s="19"/>
       <c r="J19" s="297"/>
       <c r="K19" s="297"/>
-      <c r="M19" s="337" t="s">
+      <c r="M19" s="335" t="s">
         <v>225</v>
       </c>
       <c r="N19" s="336"/>
       <c r="O19" s="336"/>
-      <c r="Q19" s="337" t="s">
+      <c r="Q19" s="335" t="s">
         <v>226</v>
       </c>
       <c r="R19" s="336"/>
@@ -45429,7 +45431,7 @@
       <c r="T19" s="298" t="s">
         <v>227</v>
       </c>
-      <c r="U19" s="337" t="s">
+      <c r="U19" s="335" t="s">
         <v>217</v>
       </c>
       <c r="V19" s="336"/>
@@ -45457,17 +45459,17 @@
       <c r="I20" s="29"/>
       <c r="J20" s="299"/>
       <c r="K20" s="299"/>
-      <c r="M20" s="335" t="s">
+      <c r="M20" s="339" t="s">
         <v>218</v>
       </c>
       <c r="N20" s="336"/>
       <c r="O20" s="336"/>
-      <c r="Q20" s="335" t="s">
+      <c r="Q20" s="339" t="s">
         <v>218</v>
       </c>
       <c r="R20" s="336"/>
       <c r="S20" s="336"/>
-      <c r="U20" s="335" t="s">
+      <c r="U20" s="339" t="s">
         <v>218</v>
       </c>
       <c r="V20" s="336"/>
@@ -47414,34 +47416,34 @@
     <row r="57" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="58" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="59" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="321" t="s">
+      <c r="A59" s="317" t="s">
         <v>119</v>
       </c>
-      <c r="B59" s="320"/>
-      <c r="C59" s="322"/>
+      <c r="B59" s="316"/>
+      <c r="C59" s="318"/>
       <c r="D59" s="305"/>
       <c r="E59" s="305"/>
-      <c r="F59" s="319"/>
-      <c r="G59" s="320"/>
-      <c r="H59" s="323"/>
-      <c r="I59" s="322"/>
+      <c r="F59" s="315"/>
+      <c r="G59" s="316"/>
+      <c r="H59" s="319"/>
+      <c r="I59" s="318"/>
       <c r="J59" s="306"/>
       <c r="K59" s="306"/>
-      <c r="M59" s="321" t="s">
+      <c r="M59" s="317" t="s">
         <v>119</v>
       </c>
-      <c r="N59" s="320"/>
-      <c r="O59" s="322"/>
-      <c r="Q59" s="321" t="s">
+      <c r="N59" s="316"/>
+      <c r="O59" s="318"/>
+      <c r="Q59" s="317" t="s">
         <v>119</v>
       </c>
-      <c r="R59" s="320"/>
-      <c r="S59" s="322"/>
-      <c r="U59" s="321" t="s">
+      <c r="R59" s="316"/>
+      <c r="S59" s="318"/>
+      <c r="U59" s="317" t="s">
         <v>119</v>
       </c>
-      <c r="V59" s="320"/>
-      <c r="W59" s="322"/>
+      <c r="V59" s="316"/>
+      <c r="W59" s="318"/>
     </row>
     <row r="60" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="14" t="s">
@@ -47469,17 +47471,17 @@
       </c>
       <c r="J60" s="105"/>
       <c r="K60" s="105"/>
-      <c r="M60" s="337" t="s">
+      <c r="M60" s="335" t="s">
         <v>225</v>
       </c>
       <c r="N60" s="336"/>
       <c r="O60" s="336"/>
-      <c r="Q60" s="337" t="s">
+      <c r="Q60" s="335" t="s">
         <v>226</v>
       </c>
       <c r="R60" s="336"/>
       <c r="S60" s="336"/>
-      <c r="U60" s="337" t="s">
+      <c r="U60" s="335" t="s">
         <v>217</v>
       </c>
       <c r="V60" s="336"/>
@@ -48500,34 +48502,34 @@
       <c r="K84" s="2"/>
     </row>
     <row r="85" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="321" t="s">
+      <c r="A85" s="317" t="s">
         <v>154</v>
       </c>
-      <c r="B85" s="320"/>
-      <c r="C85" s="322"/>
+      <c r="B85" s="316"/>
+      <c r="C85" s="318"/>
       <c r="D85" s="305"/>
       <c r="E85" s="305"/>
-      <c r="F85" s="319"/>
-      <c r="G85" s="320"/>
-      <c r="H85" s="323"/>
-      <c r="I85" s="322"/>
+      <c r="F85" s="315"/>
+      <c r="G85" s="316"/>
+      <c r="H85" s="319"/>
+      <c r="I85" s="318"/>
       <c r="J85" s="306"/>
       <c r="K85" s="306"/>
-      <c r="M85" s="321" t="s">
+      <c r="M85" s="317" t="s">
         <v>154</v>
       </c>
-      <c r="N85" s="320"/>
-      <c r="O85" s="322"/>
-      <c r="Q85" s="321" t="s">
+      <c r="N85" s="316"/>
+      <c r="O85" s="318"/>
+      <c r="Q85" s="317" t="s">
         <v>154</v>
       </c>
-      <c r="R85" s="320"/>
-      <c r="S85" s="322"/>
-      <c r="U85" s="321" t="s">
+      <c r="R85" s="316"/>
+      <c r="S85" s="318"/>
+      <c r="U85" s="317" t="s">
         <v>154</v>
       </c>
-      <c r="V85" s="320"/>
-      <c r="W85" s="322"/>
+      <c r="V85" s="316"/>
+      <c r="W85" s="318"/>
     </row>
     <row r="86" spans="1:23" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="34" t="s">
@@ -50190,6 +50192,21 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="U85:W85"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="Q85:S85"/>
+    <mergeCell ref="Q60:S60"/>
+    <mergeCell ref="A85:C85"/>
+    <mergeCell ref="M85:O85"/>
+    <mergeCell ref="F85:G85"/>
+    <mergeCell ref="H85:I85"/>
+    <mergeCell ref="H59:I59"/>
+    <mergeCell ref="Q59:S59"/>
+    <mergeCell ref="Q2:S2"/>
+    <mergeCell ref="M19:O19"/>
+    <mergeCell ref="U2:W2"/>
+    <mergeCell ref="Q19:S19"/>
+    <mergeCell ref="U20:W20"/>
     <mergeCell ref="U1:W1"/>
     <mergeCell ref="U19:W19"/>
     <mergeCell ref="U60:W60"/>
@@ -50206,21 +50223,6 @@
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="F3:G3"/>
     <mergeCell ref="F59:G59"/>
-    <mergeCell ref="H59:I59"/>
-    <mergeCell ref="Q59:S59"/>
-    <mergeCell ref="Q2:S2"/>
-    <mergeCell ref="M19:O19"/>
-    <mergeCell ref="U2:W2"/>
-    <mergeCell ref="Q19:S19"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="Q85:S85"/>
-    <mergeCell ref="Q60:S60"/>
-    <mergeCell ref="A85:C85"/>
-    <mergeCell ref="M85:O85"/>
-    <mergeCell ref="F85:G85"/>
-    <mergeCell ref="H85:I85"/>
-    <mergeCell ref="U20:W20"/>
-    <mergeCell ref="U85:W85"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -50243,11 +50245,11 @@
       <c r="A2" s="310"/>
       <c r="B2" s="311">
         <f>Balance!F3</f>
-        <v>2</v>
+        <v>2025</v>
       </c>
       <c r="C2" s="311" t="str">
         <f>Balance!H3</f>
-        <v>3 (INCORRECTO)</v>
+        <v>2026 (INCORRECTO)</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">

</xml_diff>